<commit_message>
Correct PAYE statutory deduction calculations
</commit_message>
<xml_diff>
--- a/resources/paye-calculation-template.xlsx
+++ b/resources/paye-calculation-template.xlsx
@@ -115,7 +115,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -172,6 +172,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -563,7 +566,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -607,7 +609,6 @@
       </c>
       <c r="B8" s="5" t="inlineStr"/>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -708,30 +709,32 @@
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Employee NSSF contribution</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>0</v>
+          <t>NSSF employee contribution (6% of gross)</t>
+        </is>
+      </c>
+      <c r="B17" s="20">
+        <f>B24*6%</f>
+        <v/>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Enter actual employee NSSF contribution</t>
+          <t>Non-taxable deduction in this template: 6% of gross cash pay.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>SHIF contribution</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="n">
-        <v>0</v>
+          <t>SHA contribution (2.75% of gross)</t>
+        </is>
+      </c>
+      <c r="B18" s="20">
+        <f>B24*2.75%</f>
+        <v/>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Enter employee SHIF contribution</t>
+          <t>Non-taxable deduction in this template: 2.75% of gross cash pay.</t>
         </is>
       </c>
     </row>
@@ -780,7 +783,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
@@ -823,7 +825,7 @@
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Affordable Housing Levy deduction</t>
+          <t>Affordable Housing Levy (1.5% of gross)</t>
         </is>
       </c>
       <c r="B26" s="10">
@@ -832,23 +834,23 @@
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Template assumption: 1.5% of gross cash pay; confirm applicable basis</t>
+          <t>Non-taxable deduction in this template: 1.5% of gross cash pay.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Allowable pension deduction</t>
+          <t>Allowable pension deduction + NSSF</t>
         </is>
       </c>
       <c r="B27" s="10">
-        <f>MIN(B16,30000)</f>
+        <f>MIN(B16,30000)+B17</f>
         <v/>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>KRA monthly cap used in this template</t>
+          <t>Employee pension contribution plus NSSF deduction; pension cap applies only to B16.</t>
         </is>
       </c>
     </row>
@@ -887,7 +889,7 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>SHIF deduction</t>
+          <t>SHA deduction</t>
         </is>
       </c>
       <c r="B30" s="10">
@@ -896,26 +898,30 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Enter the applicable employee contribution</t>
+          <t>2.75% of gross cash pay; treated as non-taxable deduction in this template.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
         <is>
-          <t>Total allowable deductions</t>
+          <t>Total non-taxable / allowable deductions</t>
         </is>
       </c>
       <c r="B31" s="12">
         <f>SUM(B26:B30)</f>
         <v/>
       </c>
-      <c r="C31" s="13" t="inlineStr"/>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>Includes Housing Levy, pension, NSSF, mortgage interest, post-retirement medical, and SHA.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>Taxable pay</t>
+          <t>Taxable pay after non-taxable deductions</t>
         </is>
       </c>
       <c r="B32" s="12">
@@ -1051,7 +1057,7 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>NSSF employee contribution</t>
+          <t>NSSF employee contribution (6% of gross)</t>
         </is>
       </c>
       <c r="B42" s="10">
@@ -1060,7 +1066,7 @@
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Entered manually; confirm current NSSF tier contribution</t>
+          <t>Non-taxable payroll deduction.</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1089,7 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>SHIF contribution</t>
+          <t>SHA contribution (2.75% of gross)</t>
         </is>
       </c>
       <c r="B44" s="10">
@@ -1092,14 +1098,14 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Actual payroll deduction</t>
+          <t>Non-taxable payroll deduction.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Affordable Housing Levy</t>
+          <t>Affordable Housing Levy (1.5% of gross)</t>
         </is>
       </c>
       <c r="B45" s="10">
@@ -1108,7 +1114,7 @@
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Employee deduction</t>
+          <t>Non-taxable payroll deduction.</t>
         </is>
       </c>
     </row>
@@ -1124,16 +1130,14 @@
       </c>
       <c r="C46" s="13" t="inlineStr">
         <is>
-          <t>Cash pay less PAYE and employee deductions</t>
-        </is>
-      </c>
-    </row>
-    <row r="47"/>
-    <row r="48"/>
+          <t>Gross cash pay less PAYE, NSSF, pension, SHA, and Housing Levy.</t>
+        </is>
+      </c>
+    </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Important: non-cash benefits are included in taxable income but are not added to estimated cash pay.</t>
+          <t>Statutory deductions in this template: NSSF 6%, SHA 2.75%, and Affordable Housing Levy 1.5% of gross cash pay. They are deducted before PAYE and from net cash pay.</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1220,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
         <is>
@@ -1244,53 +1247,63 @@
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>3. Enter deductions</t>
+          <t>3. Statutory deductions</t>
         </is>
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>Enter actual employee pension, NSSF, SHIF, mortgage-interest, post-retirement medical, and qualifying insurance premium amounts.</t>
+          <t>NSSF, SHA, and Housing Levy are calculated automatically from gross cash pay using 6%, 2.75%, and 1.5% respectively, then deducted before PAYE.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>4. Review formulas</t>
+          <t>4. Other deductions</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>The workbook applies the KRA monthly PAYE bands, personal relief, selected allowable deduction caps, and insurance relief shown on the Rates &amp; Sources sheet.</t>
+          <t>Enter pension, mortgage-interest, post-retirement medical, and insurance-premium inputs where applicable.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>5. Review special cases</t>
+          <t>5. Review formulas</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Benefits, expatriate/non-resident employment, pension arrangements, housing, bonuses, and statutory deductions can require specific treatment.</t>
+          <t>The workbook applies the KRA monthly PAYE bands, personal relief, deduction caps, and insurance relief shown on the Rates &amp; Sources sheet.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>6. File and remit</t>
+          <t>6. Review special cases</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
+          <t>Benefits, expatriate/non-resident employment, pension arrangements, bonuses, and statutory deduction limits can require specific treatment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>7. File and remit</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Use the final PAYE figure as a preparation aid only. Reconcile to payroll records and file/remit through the applicable KRA process.</t>
         </is>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
@@ -1299,7 +1312,6 @@
       </c>
     </row>
     <row r="12"/>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
@@ -1330,7 +1342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1346,7 +1358,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1479,7 +1490,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
         <is>
@@ -1510,65 +1520,86 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>1.5% employee</t>
+          <t>1.5% of gross</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>1.5% employer</t>
+          <t>Employee and employer</t>
         </is>
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>Template calculates employee amount on gross cash pay; confirm applicable basis</t>
+          <t>Non-taxable deduction assumption used in workbook</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
         <is>
-          <t>Insurance relief</t>
+          <t>NSSF employee contribution</t>
         </is>
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>15% of premiums</t>
+          <t>6% of gross</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>Maximum KES 60,000/year</t>
+          <t>Employee contribution</t>
         </is>
       </c>
       <c r="D12" s="17" t="inlineStr">
         <is>
-          <t>Monthly cap in workbook: KES 5,000</t>
+          <t>Non-taxable deduction assumption used in workbook</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
         <is>
-          <t>Deduction caps</t>
+          <t>SHA contribution</t>
         </is>
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
+          <t>2.75% of gross</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Employee contribution</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>Non-taxable deduction assumption used in workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Other deduction caps</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>Pension KES 30,000/month</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Mortgage KES 30,000/month</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Post-retirement medical KES 15,000/month</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
@@ -1612,8 +1643,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
@@ -1626,9 +1655,22 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Version note</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Corrected September 2026: NSSF 6%, SHA 2.75%, and Housing Levy 1.5% are calculated on gross cash pay and treated as non-taxable deductions in this template. Confirm statutory bases and limits before filing.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B22:D22"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="B21:D21"/>

</xml_diff>